<commit_message>
data backup + FII/DII refresh (2026-06-18)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I553"/>
+  <dimension ref="A1:I554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26315,6 +26315,53 @@
         </is>
       </c>
       <c r="I553" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>14806.3</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>14704.71</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>101.59</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>16611.87</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>15050.47</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>1561.4</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-06-19)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I553"/>
+  <dimension ref="A1:I555"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26315,6 +26315,100 @@
         </is>
       </c>
       <c r="I553" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>14806.3</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>14704.71</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>101.59</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>16611.87</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>15050.47</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>1561.4</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>14611.83</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>15637.03</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>-1025.2</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>16163.18</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>12646.37</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>3516.81</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-20)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I555"/>
+  <dimension ref="A1:I574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26409,6 +26409,899 @@
         </is>
       </c>
       <c r="I555" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>10082.08</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>10717.99</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>-635.91</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>17391.78</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>16356.06</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>1035.72</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>15396.07</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>15378.21</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>17.86</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>16863.04</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>16182.83</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>680.21</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>16744.73</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>18588.13</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>-1843.4</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>17274.01</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>13636.75</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>3637.26</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>18988.03</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>18604.27</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>383.76</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>24844.03</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>19096.28</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>5747.75</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>24754.26</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>26104.36</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>-1350.1</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>55273.85</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>52472.4</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>2801.45</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>23273.71</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>25830.46</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>-2556.75</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>23432.58</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>16590.24</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>6842.34</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>11623.31</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>12763.81</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>-1140.5</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>17136.57</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>13977.33</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>3159.24</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>14018.4</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>14330.22</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>-311.82</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>17391.61</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>15607.21</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>1784.4</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>13337.33</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>11982.0</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>1355.33</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>18676.35</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>20630.24</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>-1953.89</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>11686.1</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>11443.07</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>243.03</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>19727.56</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>15936.14</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>3791.42</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>18414.01</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>18020.82</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>393.19</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>18897.44</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>19280.87</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>-383.43</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>17463.95</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>15501.15</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>1962.8</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>19165.13</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>18374.97</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>790.16</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>14388.41</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>14921.27</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>-532.86</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>18302.87</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>16245.08</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>2057.79</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>15318.07</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>12714.35</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>2603.72</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>17171.75</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>15152.07</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>2019.68</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>10386.48</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>13448.75</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>-3062.27</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>17393.46</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>15221.76</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>2171.7</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>12763.43</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>13503.12</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>-739.69</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>20420.87</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>17493.16</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>2927.71</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>13207.46</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>13943.29</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>-735.83</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>16226.42</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>15521.49</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>704.93</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>13576.08</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>17781.64</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>-4205.56</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>19236.8</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>16250.39</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>2986.41</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>14393.77</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>14770.18</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>-376.41</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>17180.08</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>16162.19</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>1017.89</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-21)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I574"/>
+  <dimension ref="A1:I575"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27302,6 +27302,53 @@
         </is>
       </c>
       <c r="I574" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>13312.67</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>14433.71</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>-1121.04</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>16187.84</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>14875.81</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>1312.03</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-22)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I575"/>
+  <dimension ref="A1:I576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27349,6 +27349,53 @@
         </is>
       </c>
       <c r="I575" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>16327.88</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>14677.72</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>1650.16</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>14638.54</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>15295.42</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>-656.88</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-24)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I576"/>
+  <dimension ref="A1:I578"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27396,6 +27396,100 @@
         </is>
       </c>
       <c r="I576" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>12889.82</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>13709.02</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>-819.2</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>13665.69</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>14083.95</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>-418.26</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>11472.08</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>14471.31</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>-2999.23</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>16575.3</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>13628.16</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>2947.14</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-27)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I578"/>
+  <dimension ref="A1:I579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27490,6 +27490,53 @@
         </is>
       </c>
       <c r="I578" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>11123.86</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>15016.63</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>-3892.77</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>18959.43</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>13505.88</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>5453.55</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-28): CSV -> 2026-07-27 (+1 day, 579 days); IPO & Brent snapshots refreshed
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I579"/>
+  <dimension ref="A1:I580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27537,6 +27537,53 @@
         </is>
       </c>
       <c r="I579" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>11695.95</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>13384.18</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>-1688.23</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>15937.1</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>13607.96</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>2329.14</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-29)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I580"/>
+  <dimension ref="A1:I581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27584,6 +27584,53 @@
         </is>
       </c>
       <c r="I580" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>17530.97</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>16775.64</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>755.33</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>18256.88</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>16592.72</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>1664.16</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-30)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I581"/>
+  <dimension ref="A1:I582"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27631,6 +27631,53 @@
         </is>
       </c>
       <c r="I581" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>17358.31</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>14376.44</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>2981.87</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>18176.22</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>17178.2</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>998.02</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-07-31)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I582"/>
+  <dimension ref="A1:I583"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27678,6 +27678,53 @@
         </is>
       </c>
       <c r="I582" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>17431.96</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>13808.45</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>3623.51</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>17979.63</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>19843.66</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>-1864.03</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-01)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I583"/>
+  <dimension ref="A1:I584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27725,6 +27725,53 @@
         </is>
       </c>
       <c r="I583" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>19045.51</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>18768.03</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>277.48</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>19885.8</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>17625.43</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>2260.37</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-04)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I584"/>
+  <dimension ref="A1:I585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27772,6 +27772,53 @@
         </is>
       </c>
       <c r="I584" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>12621.89</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>11699.63</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>922.26</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>18325.97</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>16754.79</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>1571.18</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-05)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I585"/>
+  <dimension ref="A1:I586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27819,6 +27819,53 @@
         </is>
       </c>
       <c r="I585" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>15630.45</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>13183.98</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>2446.47</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>15241.39</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>16177.53</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>-936.14</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-06)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I586"/>
+  <dimension ref="A1:I587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27866,6 +27866,53 @@
         </is>
       </c>
       <c r="I586" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>15940.5</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>16883.92</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>-943.42</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>19353.43</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>16470.26</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>2883.17</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-07)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I587"/>
+  <dimension ref="A1:I588"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27913,6 +27913,53 @@
         </is>
       </c>
       <c r="I587" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>16161.35</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>16179.21</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>-17.86</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>19723.68</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>15710.08</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>4013.6</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-10)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I588"/>
+  <dimension ref="A1:I589"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27960,6 +27960,53 @@
         </is>
       </c>
       <c r="I588" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>12941.31</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>12461.07</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>480.24</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>15679.58</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>15444.02</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>235.56</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-11)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I589"/>
+  <dimension ref="A1:I590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28007,6 +28007,53 @@
         </is>
       </c>
       <c r="I589" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>13161.56</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>11186.8</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>1974.76</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>15868.51</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>17158.8</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>-1290.29</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-12)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I590"/>
+  <dimension ref="A1:I591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28054,6 +28054,53 @@
         </is>
       </c>
       <c r="I590" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>14628.47</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>14369.92</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>258.55</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>15006.72</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>14981.95</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>24.77</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-13)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I591"/>
+  <dimension ref="A1:I592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28101,6 +28101,53 @@
         </is>
       </c>
       <c r="I591" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>16584.64</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>17587.14</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>-1002.5</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>21518.55</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>15676.89</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>5841.66</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-15)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I592"/>
+  <dimension ref="A1:I594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28148,6 +28148,100 @@
         </is>
       </c>
       <c r="I592" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>14492.46</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>15003.15</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>-510.69</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>16565.14</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>12212.05</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>4353.09</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>12854.44</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>12346.32</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>508.12</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>14295.49</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>13939.09</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>356.4</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-18)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I594"/>
+  <dimension ref="A1:I595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28242,6 +28242,53 @@
         </is>
       </c>
       <c r="I594" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>11546.16</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>14081.26</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>-2535.1</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>16654.08</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>11552.62</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>5101.46</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-19)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I595"/>
+  <dimension ref="A1:I596"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28289,6 +28289,53 @@
         </is>
       </c>
       <c r="I595" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>13543.3</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>11891.77</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>1651.53</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>15566.07</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>12986.76</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>2579.31</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-20)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I596"/>
+  <dimension ref="A1:I597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28336,6 +28336,53 @@
         </is>
       </c>
       <c r="I596" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>12875.76</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>12467.77</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>407.99</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>17288.58</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>13314.86</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>3973.72</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-21)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I597"/>
+  <dimension ref="A1:I598"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28383,6 +28383,53 @@
         </is>
       </c>
       <c r="I597" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>11411.73</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>11995.09</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>-583.36</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>16932.72</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>13395.01</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>3537.71</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-24)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I598"/>
+  <dimension ref="A1:I599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28430,6 +28430,53 @@
         </is>
       </c>
       <c r="I598" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>12560.91</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>13103.62</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>-542.71</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>15258.71</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>13134.57</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>2124.14</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-25)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I599"/>
+  <dimension ref="A1:I600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28477,6 +28477,53 @@
         </is>
       </c>
       <c r="I599" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>12332.64</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>11150.98</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>1181.66</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>15337.18</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>12843.77</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>2493.41</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-26)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I600"/>
+  <dimension ref="A1:I601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28524,6 +28524,53 @@
         </is>
       </c>
       <c r="I600" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>13259.03</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>11665.5</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>1593.53</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>14280.18</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>14049.92</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>230.26</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-27)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I601"/>
+  <dimension ref="A1:I602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28571,6 +28571,53 @@
         </is>
       </c>
       <c r="I601" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>17520.49</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>17017.86</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>502.63</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>17710.07</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>11284.91</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>6425.16</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-28)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I602"/>
+  <dimension ref="A1:I603"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28618,6 +28618,53 @@
         </is>
       </c>
       <c r="I602" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>15276.94</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>15575.2</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>-298.26</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>19605.6</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>14628.43</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>4977.17</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-08-31)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I603"/>
+  <dimension ref="A1:I604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28665,6 +28665,53 @@
         </is>
       </c>
       <c r="I603" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>13263.62</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>18303.42</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>-5039.8</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>16539.38</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>11355.45</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>5183.93</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-01)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I604"/>
+  <dimension ref="A1:I605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28712,6 +28712,53 @@
         </is>
       </c>
       <c r="I604" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>60025.88</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>68011.76</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>-7985.88</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>19730.38</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>15141.5</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>4588.88</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-02)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I605"/>
+  <dimension ref="A1:I606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28759,6 +28759,53 @@
         </is>
       </c>
       <c r="I605" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>17807.53</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>16664.15</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>1143.38</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>15635.49</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>13788.55</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>1846.94</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-03)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I606"/>
+  <dimension ref="A1:I607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28806,6 +28806,53 @@
         </is>
       </c>
       <c r="I606" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>26715.88</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>20027.51</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>6688.37</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>17639.89</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>14826.91</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>2812.98</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-04)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I607"/>
+  <dimension ref="A1:I608"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28853,6 +28853,53 @@
         </is>
       </c>
       <c r="I607" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>13596.04</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>15941.91</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>-2345.87</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>17063.65</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>12086.19</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>4977.46</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-05)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I608"/>
+  <dimension ref="A1:I609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28900,6 +28900,53 @@
         </is>
       </c>
       <c r="I608" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>13857.58</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>16969.52</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>-3111.94</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>19254.19</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>10324.07</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>8930.12</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-08)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I609"/>
+  <dimension ref="A1:I610"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28947,6 +28947,53 @@
         </is>
       </c>
       <c r="I609" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>9581.19</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>9301.06</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>280.13</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>13154.13</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>12587.37</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>566.76</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>